<commit_message>
Complete colleague discovery experience
- Add searchable colleague navigation with smooth camera focusing
- Add anchored hover and selected profile information popups
- Extend public-safe profile data fields and record the viewer state
</commit_message>
<xml_diff>
--- a/project/instance_template/boatboard.xlsx
+++ b/project/instance_template/boatboard.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="R2bcc58ad1acf4e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="Re659cc86edfc4aba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R5a70ca1fd759426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="R1146bc431c614625"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="R5e5068d13d9640ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R3c04a43fe40f4e76"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -442,6 +442,9 @@
     <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="54" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -453,6 +456,9 @@
       <x:c r="D1" s="3"/>
       <x:c r="E1" s="3"/>
       <x:c r="F1" s="3"/>
+      <x:c r="G1" s="3"/>
+      <x:c r="H1" s="3"/>
+      <x:c r="I1" s="3"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="6" t="str">
@@ -470,8 +476,17 @@
       <x:c r="E3" s="11" t="str">
         <x:v>role</x:v>
       </x:c>
-      <x:c r="F3" s="7" t="str">
+      <x:c r="F3" s="11" t="str">
         <x:v>notes</x:v>
+      </x:c>
+      <x:c r="G3" s="11" t="str">
+        <x:v>whatsapp</x:v>
+      </x:c>
+      <x:c r="H3" s="11" t="str">
+        <x:v>discord</x:v>
+      </x:c>
+      <x:c r="I3" s="7" t="str">
+        <x:v>description</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -491,10 +506,13 @@
       <x:c r="F4" s="12" t="str">
         <x:v>Delete this example row when adding real colleagues</x:v>
       </x:c>
+      <x:c r="G4" s="12" t="str"/>
+      <x:c r="H4" s="12" t="str"/>
+      <x:c r="I4" s="12" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
+    <x:mergeCell ref="A1:I1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Prepare generic BoatBoard repository
- replace company-specific defaults with reusable BoatBoard seed data
- document the local private-instance boundary and remote backup state
- add the application preview for the project repository
</commit_message>
<xml_diff>
--- a/project/instance_template/boatboard.xlsx
+++ b/project/instance_template/boatboard.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="R1146bc431c614625"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="R5e5068d13d9640ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R3c04a43fe40f4e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="R995df94d07fd4583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="R17c3b01b66ff4da4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R9a4dfb08d0804309"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -352,7 +352,7 @@
         <x:v>company_name</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Eduzz</x:v>
+        <x:v>BoatBoard</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>

<commit_message>
Deliver standalone local BoatBoard MVP
- add reproducible Windows executable export with clean first-run data
- align viewer/editor interactions and layered popup behavior
- document the local instance boundary and future hosted integration path
</commit_message>
<xml_diff>
--- a/project/instance_template/boatboard.xlsx
+++ b/project/instance_template/boatboard.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="R995df94d07fd4583"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="R17c3b01b66ff4da4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R9a4dfb08d0804309"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="R98669aa22c17478c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="R2f55803d245347d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R6363c51ddda24e50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -414,15 +414,9 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="12" t="str">
-        <x:v>team-example</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>Example Team</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
-        <x:v>Delete this example row when adding real teams</x:v>
-      </x:c>
+      <x:c r="A4" s="12"/>
+      <x:c r="B4" s="12"/>
+      <x:c r="C4" s="12"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -490,25 +484,15 @@
       </x:c>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="12" t="str">
-        <x:v>person-example</x:v>
-      </x:c>
-      <x:c r="B4" s="12" t="str">
-        <x:v>Example Person</x:v>
-      </x:c>
-      <x:c r="C4" s="12" t="str">
-        <x:v>team-example</x:v>
-      </x:c>
-      <x:c r="D4" s="12" t="str">
-        <x:v>person-example.jpg</x:v>
-      </x:c>
-      <x:c r="E4" s="12" t="str"/>
-      <x:c r="F4" s="12" t="str">
-        <x:v>Delete this example row when adding real colleagues</x:v>
-      </x:c>
-      <x:c r="G4" s="12" t="str"/>
-      <x:c r="H4" s="12" t="str"/>
-      <x:c r="I4" s="12" t="str"/>
+      <x:c r="A4" s="12"/>
+      <x:c r="B4" s="12"/>
+      <x:c r="C4" s="12"/>
+      <x:c r="D4" s="12"/>
+      <x:c r="E4" s="12"/>
+      <x:c r="F4" s="12"/>
+      <x:c r="G4" s="12"/>
+      <x:c r="H4" s="12"/>
+      <x:c r="I4" s="12"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Unify responsive viewer and editor behavior
- Consolidate wide, compact desktop, and touch presentations around shared responsive foundations
- Refine mobile pan, zoom, popup anchoring, directory sizing, and immediate search filtering
- Add editor marquee movement, board-title editing, runtime identification, and generic BoatTitle seed
- Preserve private instance data outside Git and refresh durable project guidance
</commit_message>
<xml_diff>
--- a/project/instance_template/boatboard.xlsx
+++ b/project/instance_template/boatboard.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="R98669aa22c17478c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="R2f55803d245347d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R6363c51ddda24e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company" sheetId="1" r:id="Rc77b1981e8494ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="2" r:id="R396bbdfb8c504179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Colleagues" sheetId="3" r:id="R7a88145e21794ab5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -352,7 +352,7 @@
         <x:v>company_name</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>BoatBoard</x:v>
+        <x:v>BoatTitle</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -360,7 +360,7 @@
         <x:v>page_title</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Boat Board</x:v>
+        <x:v>BoatTitle</x:v>
       </x:c>
     </x:row>
     <x:row r="7">

</xml_diff>